<commit_message>
possibilidade de apagar eventos antes
</commit_message>
<xml_diff>
--- a/output/forro_agenda_2026-03-24.xlsx
+++ b/output/forro_agenda_2026-03-24.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Godoferdo (408n)</t>
+          <t>Godofredo (408n)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Xinela - Meriele e sua gente, DJ Dark Lion</t>
+          <t>Xinela da - Meriele e sua gente, DJ Dark Lion</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>R$20 - R$35</t>
+          <t>R$20-35</t>
         </is>
       </c>
     </row>
@@ -676,13 +676,12 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Ispilucite - Forró Legal
-DJ Tiago Braga</t>
+          <t>DJ Tiago Braga</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>R$30 ~ R$50</t>
+          <t>R$30</t>
         </is>
       </c>
     </row>
@@ -714,12 +713,12 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Forró Sóxdó - Forró Cobogó + Inácio Botelho</t>
+          <t>Forró Sóxodó - Forró Cobogó + Inácio Botelho</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>R$0 ~ R$?</t>
+          <t>R$?</t>
         </is>
       </c>
     </row>
@@ -751,14 +750,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Baile do Ipê - Ipê Fulô
-DJ Breno Borro
-Contribuição voluntária (sugestão R$15)</t>
+          <t>Baile do Ipê - Ipê Fulô, DJ Breno Borro</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>R$??</t>
+          <t>contribuição voluntária</t>
         </is>
       </c>
     </row>
@@ -795,14 +792,14 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>R$18 ~ R$35 (meia)</t>
+          <t>R$18</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Extraído em: 24/03/2026 19:51</t>
+          <t>Extraído em: 24/03/2026 20:15</t>
         </is>
       </c>
     </row>

</xml_diff>